<commit_message>
Regenerate Section 32 direct-image submission
Co-authored-by: ryangille02 <ryangille02@aol.com>
</commit_message>
<xml_diff>
--- a/deliverables/GPT56_SOL_SECTION32_MULTI_TRACT_SPRINT_20260716/GPT56_SOL_SECTION32_IMPROVED_WORKBOOK_20260716.xlsx
+++ b/deliverables/GPT56_SOL_SECTION32_MULTI_TRACT_SPRINT_20260716/GPT56_SOL_SECTION32_IMPROVED_WORKBOOK_20260716.xlsx
@@ -12,13 +12,14 @@
     <sheet name="Title" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Runsheet" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Leases" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="WI Historical" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="WI Present Candidates" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Modern Chain" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Addresses" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Acquisition Queue" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Template Improvements" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="QA" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Acreage Reconciliation" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="WI Historical" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="WI Present Candidates" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Modern Chain" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Addresses" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Acquisition Queue" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Template Improvements" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="QA" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$H$8</definedName>
@@ -27,24 +28,26 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Tract Control'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Title'!$A$1:$R$6</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Title'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Runsheet'!$A$1:$Z$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Runsheet'!$A$1:$Z$21</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Runsheet'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Leases'!$A$1:$X$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Leases'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'WI Historical'!$A$1:$I$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'WI Historical'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'WI Present Candidates'!$A$1:$L$6</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="6">'WI Present Candidates'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Modern Chain'!$A$1:$H$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="7">'Modern Chain'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Addresses'!$A$1:$G$2</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Addresses'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Acquisition Queue'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Acquisition Queue'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Template Improvements'!$A$1:$B$11</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Template Improvements'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'QA'!$A$1:$C$12</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="11">'QA'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Acreage Reconciliation'!$A$1:$C$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Acreage Reconciliation'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'WI Historical'!$A$1:$I$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'WI Historical'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'WI Present Candidates'!$A$1:$L$2</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="7">'WI Present Candidates'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Modern Chain'!$A$1:$H$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="8">'Modern Chain'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Addresses'!$A$1:$G$16</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="9">'Addresses'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Acquisition Queue'!$A$1:$D$8</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Acquisition Queue'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Template Improvements'!$A$1:$B$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Template Improvements'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'QA'!$A$1:$C$14</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="12">'QA'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -588,6 +591,623 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="41" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Party</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Recorded Address</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Normalized Address</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Address Type</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Effective/Recording Date</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Currentness Caveat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Diversified Production LLC</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>1600 Corporate Drive, Birmingham, AL 35242</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>1600 Corporate Drive, Birmingham, AL 35242</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Recorded instrument address</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>2395/415–464; 2400/551–567</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2022-11-18 / 2023-03-02</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Historic recorded address; not represented as verified current</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Cora B. Garrett; S.A. Garrett</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mayfield, Oklahoma</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Mayfield, OK</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Lessor locality</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>OGL 63/33 / Image 0353</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>1947-11-13</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Charlie B. Crook; Ima Pearl Crook</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Route 1, Mayfield, Oklahoma</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Route 1, Mayfield, OK</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>OGL 264/345 / Image 1197</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>1972-02-05</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Cora B. LeGrand</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Sweetwater, Oklahoma</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Sweetwater, OK</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Lessor locality</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>OGL 307/31 / Image 1372</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1976-04-29</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>LaFortune co-trustees</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Bank Building, Tulsa, Oklahoma</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Bank Building, Tulsa, OK</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>OGL 340/302 / Image 1522</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>1977-10-14</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Gertrude LaFortune</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Building, Tulsa, Oklahoma 74119</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Building, Tulsa, OK 74119</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>OGL 340/304 / Image 1524</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>1977-10-14</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>George T. Harrison Jr.; Renata Harrison</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>201 North Charles Street, Baltimore, Maryland 21201</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>201 North Charles Street, Baltimore, MD 21201</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>OGL 340/323 / Image 1526</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>1977-09-29</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Carol Seidenbach Leach</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>c/o Mrs. J. Leslie Seidenbach, 2827 South Birmingham Place, Tulsa, Oklahoma</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>c/o Mrs. J. Leslie Seidenbach, 2827 South Birmingham Place, Tulsa, OK</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>OGL 342/564 / Image 1542</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>1977-09-29</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Cynthia Seidenbach Kruse</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>c/o M. B. Johnson, 1623 S. College, Tulsa, Oklahoma 74104</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>c/o M. B. Johnson, 1623 S. College, Tulsa, OK 74104</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>OGL 342/566 / Image 1544</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>1977-11-01</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>F.L. Randel</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>P. O. Box 7, c/o Ramada Inn, Big Spring, Texas 79720</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>P.O. Box 7, c/o Ramada Inn, Big Spring, TX 79720</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>OGL 352/719 / Image 1552</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>1978-05-16</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>J.L. Randel</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Box 2609, Wichita Falls, Texas</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>P.O. Box 2609, Wichita Falls, TX</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Lessor address</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>OGL 352/721 / Image 1554</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>1978-05-16</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Great Western Oil &amp; Gas, Inc.</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>4010 Palos Verdes Drive North, Suite 206, Rolling Hills Estates, California 90274</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>4010 Palos Verdes Drive N, Suite 206, Rolling Hills Estates, CA 90274</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Lessor corporate address</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>OGL 376/369 / Image 1569</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>1979-03-21</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>P. O. Box 3100, Midland, Texas 79702</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>P.O. Box 3100, Midland, TX 79702</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Assignor address</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Bk 872/Pg 279 / Image 4388</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>1985-10-29</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Leede Exploration</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>600 North Marienfeld, Midland, Texas 79701</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>600 N Marienfeld, Midland, TX 79701</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Assignee address</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Bk 872/Pg 279 / Image 4388</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>1985-10-29</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Consolidation of Leede Trusts</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>600 North Marienfeld, Midland, Texas 79701</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>600 N Marienfeld, Midland, TX 79701</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Assignor address</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Bk 1014/Pg 75 / Image 4893</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>1988-02-18</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>Historical only; not a current mailing address</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -650,12 +1270,12 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Original OGL 63/33 plus amendments, ratifications, releases, production and shut-in records</t>
+          <t>Amendments, ratifications, releases, production and shut-in records for OGL 63/33</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Determines Pearl lease terms, status, and HBP</t>
+          <t>Determines Pearl lease continuation, status, and HBP beyond the reviewed original face</t>
         </is>
       </c>
     </row>
@@ -690,12 +1310,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Complete 872/279, unrecorded 1984 agreement, and every scheduled OGL</t>
+          <t>Missing 872/279 pages 280–281, unrecorded 1984 agreement, amendments, releases, and HBP records</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Enables lease matrix, overlap/gap analysis, and burden review</t>
+          <t>Completes assignment terms and current-effect review beyond the faces and exhibits already inspected</t>
         </is>
       </c>
     </row>
@@ -766,7 +1386,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -898,13 +1518,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -959,7 +1579,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>All scopes marked non-additive; T4/T5 nominal acres intentionally blank</t>
+          <t>T4 document-location math is separately labeled: 1,360 row / 560 unique / 800 overlap / 80 schedule gap; no current net acres</t>
         </is>
       </c>
     </row>
@@ -1027,14 +1647,14 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Only one recorded Diversified address included</t>
+          <t>One modern recorded Diversified address and 14 exact historical addresses; every historical address is marked not current</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Formula safeguards</t>
+          <t>Original OGL faces</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1044,14 +1664,14 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>No ownership-total formula exists; no blank-to-zero arithmetic</t>
+          <t>Eleven lease faces reviewed at Images 0353, 1197–1198, 1372, 1522–1527, 1542–1545, 1552–1555, 1569–1570</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Stale template facts</t>
+          <t>Face/index conflicts visible</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1061,14 +1681,14 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>No Section 27, Cherokee, Kunu, Greenhead, Aztek, or Phillips facts imported</t>
+          <t>352/719: 5169 vs 5051; 352/721: 5168 vs 5052; 376/369: 3757 vs 3707</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Index limitation</t>
+          <t>Formula safeguards</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1078,46 +1698,80 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Page 48 gap and locator-only limits disclosed</t>
+          <t>No ownership-total formula exists; no blank-to-zero arithmetic</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Drive upload reopened</t>
+          <t>Stale template facts</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Must remain OPEN until files are uploaded and reopened from Drive</t>
+          <t>No Section 27, Cherokee, Kunu, Greenhead, Aztek, or Phillips facts imported</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>Index limitation</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Page 48 gap and locator-only limits disclosed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Drive upload reopened</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Must remain OPEN until files are uploaded and reopened from Drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
           <t>Release decision</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr">
         <is>
           <t>HOLD</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Exact present mineral/lease/WI conclusions are not supported</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C12"/>
+  <autoFilter ref="A1:C14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -1302,12 +1956,12 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Overlapping lease-by-lease and depth-by-depth scope; non-additive. General assignment interval is top Morrow–19,480 feet, subject to exceptions.</t>
+          <t>Overlapping lease-by-lease and depth-by-depth scope; non-additive. Eleven listed Section 32 lease rows total 1,360 row acres but reconcile to 560 unique nominal acres, 800 overlapping row acres, and an 80-acre S/2 NW/4 schedule gap. General assignment interval is top Morrow–19,480 feet, subject to exceptions.</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Historic lease identities and assignment depth limitations are supported. Unique acreage, uncovered gaps, current lease status, and current quantum are NOT DETERMINED.</t>
+          <t>Original faces for all 11 listed leases and Bk 872/Pg 279 assignment/exhibits support the historic lease package and document-location math. Current lease status, HBP, successor title, and current quantum are NOT DETERMINED.</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -1376,8 +2030,8 @@
     <col width="42" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="36" customWidth="1" min="11" max="11"/>
-    <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="19" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
@@ -1515,12 +2169,20 @@
           <t>264/345; 352/719; 352/721; 376/369</t>
         </is>
       </c>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>1/8 at 264/345; 3/16 at later original faces</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>5 years by reviewed faces; commencement varies</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="n"/>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>Direct images + schedule references</t>
+          <t>Direct original images + recorded exhibits</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
@@ -1530,7 +2192,7 @@
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>Complete downstream fee/mineral and lease chains</t>
+          <t>Complete downstream fee/mineral, amendment, release, and HBP chains</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
@@ -1573,12 +2235,20 @@
           <t>63/33</t>
         </is>
       </c>
-      <c r="L3" s="3" t="n"/>
-      <c r="M3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>10 years from 1947-11-13</t>
+        </is>
+      </c>
       <c r="N3" s="3" t="n"/>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t>Direct image/assignment recital</t>
+          <t>Direct original image + recorded assignments</t>
         </is>
       </c>
       <c r="P3" s="3" t="inlineStr">
@@ -1588,7 +2258,7 @@
       </c>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>Pull original OGL, releases, payout and successors</t>
+          <t>Pull amendments, releases, payout, successors, and HBP evidence</t>
         </is>
       </c>
       <c r="R3" s="3" t="inlineStr">
@@ -1672,7 +2342,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>Eleven historic lease references</t>
+          <t>Eleven original OGL faces reviewed</t>
         </is>
       </c>
       <c r="H5" s="3" t="n"/>
@@ -1683,12 +2353,20 @@
           <t>Bk 872/Pg 279 schedule</t>
         </is>
       </c>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>1/8 or 3/16 by original face; later Union ORRIs are assignment-scoped</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>5 or 10 years by original face</t>
+        </is>
+      </c>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="inlineStr">
         <is>
-          <t>Partial direct-image instrument</t>
+          <t>Direct original images + assignment/exhibits</t>
         </is>
       </c>
       <c r="P5" s="3" t="inlineStr">
@@ -1698,12 +2376,12 @@
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>Pull complete assignment, agreement, OGLs, releases and HBP</t>
+          <t>Pull missing assignment pages, agreement, amendments, releases and HBP</t>
         </is>
       </c>
       <c r="R5" s="3" t="inlineStr">
         <is>
-          <t>Historic lease identities and assignment depth limitations are supported. Unique acreage, uncovered gaps, current lease status, and current quantum are NOT DETERMINED.</t>
+          <t>Original faces for all 11 listed leases and Bk 872/Pg 279 assignment/exhibits support the historic lease package and document-location math. Current lease status, HBP, successor title, and current quantum are NOT DETERMINED.</t>
         </is>
       </c>
     </row>
@@ -1784,7 +2462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:Z21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1795,19 +2473,19 @@
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
     <col width="42" customWidth="1" min="13" max="13"/>
     <col width="42" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
     <col width="42" customWidth="1" min="16" max="16"/>
     <col width="24" customWidth="1" min="17" max="17"/>
-    <col width="25" customWidth="1" min="18" max="18"/>
-    <col width="35" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="42" customWidth="1" min="19" max="19"/>
     <col width="42" customWidth="1" min="20" max="20"/>
-    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="21" max="21"/>
     <col width="12" customWidth="1" min="22" max="22"/>
     <col width="42" customWidth="1" min="23" max="23"/>
     <col width="42" customWidth="1" min="24" max="24"/>
@@ -2169,10 +2847,14 @@
           <t>1947-11-13</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>1947-11-26</t>
+        </is>
+      </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>OGL REF</t>
+          <t>OGL</t>
         </is>
       </c>
       <c r="F4" s="3" t="n"/>
@@ -2183,10 +2865,14 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>Cora B. Garrett; S.A. Garrett</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="n"/>
+          <t>Cora B. Garrett; S.A. Garrett, her husband</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Mayfield, Oklahoma</t>
+        </is>
+      </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t>C.E. McKinley</t>
@@ -2204,7 +2890,11 @@
         </is>
       </c>
       <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold face; 1/8 royalty; 10-year primary term</t>
+        </is>
+      </c>
       <c r="P4" s="3" t="n"/>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -2218,36 +2908,36 @@
       </c>
       <c r="S4" s="3" t="inlineStr">
         <is>
-          <t>DIRECT-IMAGE ASSIGNMENT RECITAL</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED ASSIGNMENT EXHIBITS</t>
         </is>
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>Bk 244/Pg 432 / Image 1062; Bk 872/Pg 284 / Image 4393</t>
+          <t>OGL 63/33 / Image 0353; Bk 244/Pg 432 / Image 1062; Bk 872/Pg 284 / Image 4393</t>
         </is>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>Images 1062, 4393</t>
+          <t>Images 0353, 1062, 4393</t>
         </is>
       </c>
       <c r="V4" s="3" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="W4" s="3" t="inlineStr">
         <is>
-          <t>Historic lease identity only</t>
+          <t>Historic lease terms and identity only</t>
         </is>
       </c>
       <c r="X4" s="3" t="n"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t>Pull original OGL and all amendments/releases</t>
+          <t>Pull amendments, ratifications, releases, pooling, production, and HBP evidence</t>
         </is>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>Royalty, term, clauses, depth, expiration, and HBP remain open.</t>
+          <t>Original face proves 1/8 royalty and 10-year term. Pooling and shut-in clauses are present but current effect, continuation, and HBP remain open.</t>
         </is>
       </c>
     </row>
@@ -2614,13 +3304,21 @@
           <t>Union Oil Company of California</t>
         </is>
       </c>
-      <c r="I8" s="3" t="n"/>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>P. O. Box 3100, Midland, Texas 79702</t>
+        </is>
+      </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
           <t>Leede Exploration</t>
         </is>
       </c>
-      <c r="K8" s="3" t="n"/>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>600 North Marienfeld, Midland, Texas 79701</t>
+        </is>
+      </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
           <t>Listed Section 32 leases; E/2 SE/4 specially limited</t>
@@ -2730,13 +3428,21 @@
           <t>Consolidation of Leede Trusts</t>
         </is>
       </c>
-      <c r="I9" s="3" t="n"/>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>600 North Marienfeld, Midland, Texas 79701</t>
+        </is>
+      </c>
       <c r="J9" s="3" t="inlineStr">
         <is>
           <t>Leede Exploration</t>
         </is>
       </c>
-      <c r="K9" s="3" t="n"/>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>600 North Marienfeld, Midland, Texas 79701</t>
+        </is>
+      </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
           <t>N/2 Section 32</t>
@@ -2752,7 +3458,11 @@
           <t>All depths below top Hunton</t>
         </is>
       </c>
-      <c r="O9" s="3" t="n"/>
+      <c r="O9" s="3" t="inlineStr">
+        <is>
+          <t>All assignor right, title, and interest in OGLs and other working/cost-bearing interests; effective for all purposes as of first production from McCall #1-29</t>
+        </is>
+      </c>
       <c r="P9" s="3" t="inlineStr">
         <is>
           <t>Royalty/ORRI reconveyance effect unclear</t>
@@ -2944,7 +3654,11 @@
           <t>Diversified Production LLC</t>
         </is>
       </c>
-      <c r="K11" s="3" t="n"/>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>1600 Corporate Drive, Birmingham, AL 35242</t>
+        </is>
+      </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
           <t>Section 32 schedule reference; asset OK48147.001.1</t>
@@ -3003,8 +3717,1120 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>1972-02-05</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>1972-02-22</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>1131</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>264/345</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>Charlie B. Crook; Ima Pearl Crook, his wife</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Route 1, Mayfield, Oklahoma</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="n"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>NE/4</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n"/>
+      <c r="O12" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 1/8; primary term 5 years commencing 1973-01-13</t>
+        </is>
+      </c>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>264/345</t>
+        </is>
+      </c>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S12" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>Images 1197–1198 and 4392. Instrument also covers 80 acres in Section 28; only 160 Section 32 row acres counted.</t>
+        </is>
+      </c>
+      <c r="U12" s="3" t="inlineStr">
+        <is>
+          <t>Images 1197–1198 and 4392</t>
+        </is>
+      </c>
+      <c r="V12" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W12" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X12" s="3" t="n"/>
+      <c r="Y12" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z12" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>1976-04-29</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>1976-06-09</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>2991</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>307/31</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Cora B. LeGrand, widow</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Sweetwater, Oklahoma</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="n"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>W/2 SE/4 and S/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="n"/>
+      <c r="O13" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 1/8; primary term 5 years commencing 1976-09-23</t>
+        </is>
+      </c>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>307/31</t>
+        </is>
+      </c>
+      <c r="R13" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S13" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T13" s="3" t="inlineStr">
+        <is>
+          <t>Images 1372 and 4391. Overlaps other listed rows; no present status or HBP inference.</t>
+        </is>
+      </c>
+      <c r="U13" s="3" t="inlineStr">
+        <is>
+          <t>Images 1372 and 4391</t>
+        </is>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W13" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X13" s="3" t="n"/>
+      <c r="Y13" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z13" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>1977-10-14</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n"/>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>340/302</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Gertrude L. LaFortune; Jeanne L. Fair; Mary Ann L. Wilcox; J.A. LaFortune Jr.; Robert J. LaFortune, co-trustees under the will of Joseph A. LaFortune</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Bank Building, Tulsa, Oklahoma</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="n"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>N/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="n"/>
+      <c r="O14" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years commencing 1977-11-28</t>
+        </is>
+      </c>
+      <c r="P14" s="3" t="n"/>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>340/302</t>
+        </is>
+      </c>
+      <c r="R14" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S14" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T14" s="3" t="inlineStr">
+        <is>
+          <t>Images 1522–1523 and 4391. Relationship to separate 340/304 remains open.</t>
+        </is>
+      </c>
+      <c r="U14" s="3" t="inlineStr">
+        <is>
+          <t>Images 1522–1523 and 4391</t>
+        </is>
+      </c>
+      <c r="V14" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W14" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X14" s="3" t="n"/>
+      <c r="Y14" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z14" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>1977-10-14</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n"/>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="n"/>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>340/304</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>Gertrude LaFortune, widow</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>2300 Fourth National Building, Tulsa, Oklahoma 74119</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="n"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>N/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="n"/>
+      <c r="O15" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years commencing 1977-11-28</t>
+        </is>
+      </c>
+      <c r="P15" s="3" t="n"/>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>340/304</t>
+        </is>
+      </c>
+      <c r="R15" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S15" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T15" s="3" t="inlineStr">
+        <is>
+          <t>Images 1524–1525 and 4391. Separate overlapping lease; do not double count.</t>
+        </is>
+      </c>
+      <c r="U15" s="3" t="inlineStr">
+        <is>
+          <t>Images 1524–1525 and 4391</t>
+        </is>
+      </c>
+      <c r="V15" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W15" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X15" s="3" t="n"/>
+      <c r="Y15" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z15" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>1977-09-29</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>1977-11-07</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n"/>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>340/323</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>George T. Harrison Jr.; Renata Harrison</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>201 North Charles Street, Baltimore, Maryland 21201</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="n"/>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>N/2 NW/4 and N/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="n"/>
+      <c r="O16" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years commencing 1977-11-27</t>
+        </is>
+      </c>
+      <c r="P16" s="3" t="n"/>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>340/323</t>
+        </is>
+      </c>
+      <c r="R16" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S16" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T16" s="3" t="inlineStr">
+        <is>
+          <t>Images 1526–1527 and 4391. This is the only listed lease aliquot covering N/2 NW/4.</t>
+        </is>
+      </c>
+      <c r="U16" s="3" t="inlineStr">
+        <is>
+          <t>Images 1526–1527 and 4391</t>
+        </is>
+      </c>
+      <c r="V16" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W16" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X16" s="3" t="n"/>
+      <c r="Y16" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z16" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>1977-09-29</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>1978-02-09</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>1089</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>342/564</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Carol Seidenbach Leach</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>c/o Mrs. J. Leslie Seidenbach, 2827 South Birmingham Place, Tulsa, Oklahoma</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="n"/>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>N/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="n"/>
+      <c r="O17" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years commencing 1977-11-30</t>
+        </is>
+      </c>
+      <c r="P17" s="3" t="n"/>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>342/564</t>
+        </is>
+      </c>
+      <c r="R17" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S17" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T17" s="3" t="inlineStr">
+        <is>
+          <t>Images 1542–1543 and 4391. Overlapping legal; current status open.</t>
+        </is>
+      </c>
+      <c r="U17" s="3" t="inlineStr">
+        <is>
+          <t>Images 1542–1543 and 4391</t>
+        </is>
+      </c>
+      <c r="V17" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W17" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X17" s="3" t="n"/>
+      <c r="Y17" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z17" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>1977-11-01</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>1978-02-09</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>1090</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>342/566</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Cynthia Seidenbach Kruse</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>c/o M. B. Johnson, 1623 S. College, Tulsa, Oklahoma 74104</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="n"/>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>N/2 SW/4</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="n"/>
+      <c r="O18" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years commencing 1977-11-30</t>
+        </is>
+      </c>
+      <c r="P18" s="3" t="n"/>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>342/566</t>
+        </is>
+      </c>
+      <c r="R18" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>Images 1544–1545 and 4391. Overlapping legal; current status open.</t>
+        </is>
+      </c>
+      <c r="U18" s="3" t="inlineStr">
+        <is>
+          <t>Images 1544–1545 and 4391</t>
+        </is>
+      </c>
+      <c r="V18" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W18" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X18" s="3" t="n"/>
+      <c r="Y18" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z18" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>1978-05-16</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>1978-06-27</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>5169</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>352/719</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>F.L. Randel</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>P. O. Box 7, c/o Ramada Inn, Big Spring, Texas 79720</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="n"/>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>NE/4</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="n"/>
+      <c r="O19" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years</t>
+        </is>
+      </c>
+      <c r="P19" s="3" t="n"/>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>352/719</t>
+        </is>
+      </c>
+      <c r="R19" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S19" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T19" s="3" t="inlineStr">
+        <is>
+          <t>Images 1552–1553 and 4391. Face instrument 5169 conflicts with protocol index 5051; clerk confirmation required.</t>
+        </is>
+      </c>
+      <c r="U19" s="3" t="inlineStr">
+        <is>
+          <t>Images 1552–1553 and 4391</t>
+        </is>
+      </c>
+      <c r="V19" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W19" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X19" s="3" t="inlineStr">
+        <is>
+          <t>Direct face instrument 5169 conflicts with protocol index 5051</t>
+        </is>
+      </c>
+      <c r="Y19" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z19" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>1978-05-16</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>1978-06-27</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>5168</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>352/721</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>J.L. Randel</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Box 2609, Wichita Falls, Texas</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="n"/>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>NE/4</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="n"/>
+      <c r="O20" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years</t>
+        </is>
+      </c>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>352/721</t>
+        </is>
+      </c>
+      <c r="R20" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>Images 1554–1555 and 4392. Face instrument 5168 conflicts with protocol index 5052; clerk confirmation required.</t>
+        </is>
+      </c>
+      <c r="U20" s="3" t="inlineStr">
+        <is>
+          <t>Images 1554–1555 and 4392</t>
+        </is>
+      </c>
+      <c r="V20" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W20" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X20" s="3" t="inlineStr">
+        <is>
+          <t>Direct face instrument 5168 conflicts with protocol index 5052</t>
+        </is>
+      </c>
+      <c r="Y20" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z20" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>T1,T4</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>1979-03-21</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>1979-04-30</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>OGL</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>3757</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>376/369</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Great Western Oil &amp; Gas, Inc., a California corporation</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>4010 Palos Verdes Drive North, Suite 206, Rolling Hills Estates, California 90274</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Union Oil Company of California</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="n"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>NE/4</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>Historic leasehold</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="n"/>
+      <c r="O21" s="3" t="inlineStr">
+        <is>
+          <t>Royalty 3/16; primary term 5 years</t>
+        </is>
+      </c>
+      <c r="P21" s="3" t="n"/>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>376/369</t>
+        </is>
+      </c>
+      <c r="R21" s="3" t="inlineStr">
+        <is>
+          <t>Union/Leede deep package</t>
+        </is>
+      </c>
+      <c r="S21" s="3" t="inlineStr">
+        <is>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
+        </is>
+      </c>
+      <c r="T21" s="3" t="inlineStr">
+        <is>
+          <t>Images 1569–1570 and 4392. Face instrument 3757 conflicts with protocol index 3707; correction metadata at 1039/20–23 remains unreviewed.</t>
+        </is>
+      </c>
+      <c r="U21" s="3" t="inlineStr">
+        <is>
+          <t>Images 1569–1570 and 4392</t>
+        </is>
+      </c>
+      <c r="V21" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="W21" s="3" t="inlineStr">
+        <is>
+          <t>Historic original lease facts only; current status OPEN</t>
+        </is>
+      </c>
+      <c r="X21" s="3" t="inlineStr">
+        <is>
+          <t>Direct face instrument 3757 conflicts with protocol index 3707</t>
+        </is>
+      </c>
+      <c r="Y21" s="3" t="inlineStr">
+        <is>
+          <t>Confirm clerk metadata; acquire amendments, corrections, releases, pooling, and HBP evidence</t>
+        </is>
+      </c>
+      <c r="Z21" s="3" t="inlineStr">
+        <is>
+          <t>Later Bk 872/Pg 279 depth and ORRI terms apply only to that assignment; they are not original-lease terms.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Z11"/>
+  <autoFilter ref="A1:Z21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
@@ -3031,16 +4857,16 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="31" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="28" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
+    <col width="42" customWidth="1" min="18" max="18"/>
     <col width="10" customWidth="1" min="19" max="19"/>
     <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
-    <col width="33" customWidth="1" min="22" max="22"/>
+    <col width="25" customWidth="1" min="21" max="21"/>
+    <col width="42" customWidth="1" min="22" max="22"/>
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="42" customWidth="1" min="24" max="24"/>
   </cols>
@@ -3175,7 +5001,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Cora B. Garrett; S.A. Garrett</t>
+          <t>Cora B. Garrett; S.A. Garrett, her husband</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -3188,7 +5014,11 @@
           <t>1947-11-13</t>
         </is>
       </c>
-      <c r="E2" s="3" t="n"/>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>1947-11-26</t>
+        </is>
+      </c>
       <c r="F2" s="3" t="n"/>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -3205,35 +5035,55 @@
       </c>
       <c r="J2" s="3" t="n"/>
       <c r="K2" s="3" t="n"/>
-      <c r="L2" s="3" t="n"/>
-      <c r="M2" s="3" t="n"/>
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>10 years</t>
+        </is>
+      </c>
       <c r="N2" s="3" t="n"/>
-      <c r="O2" s="3" t="n"/>
-      <c r="P2" s="3" t="n"/>
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>Clause present; effect not adjudicated</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Clause present; effect not adjudicated</t>
+        </is>
+      </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>244/432; 845/47; 872/279</t>
         </is>
       </c>
-      <c r="R2" s="3" t="n"/>
+      <c r="R2" s="3" t="inlineStr">
+        <is>
+          <t>Union later reserved depth-limited ORRIs in 872/279</t>
+        </is>
+      </c>
       <c r="S2" s="3" t="n"/>
       <c r="T2" s="3" t="n"/>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V2" s="3" t="inlineStr">
         <is>
-          <t>Assignment recital/direct image</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W2" s="3" t="n">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="X2" s="3" t="inlineStr">
         <is>
-          <t>Original lease and terms not reviewed</t>
+          <t>Images 0353 and 4393. Original face proves historic terms only; amendments, release, HBP, and current ownership remain open.</t>
         </is>
       </c>
     </row>
@@ -3245,7 +5095,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Charlie B. Crook; Ima Pearl Crook</t>
+          <t>Charlie B. Crook; Ima Pearl Crook, his wife</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -3283,10 +5133,14 @@
       </c>
       <c r="J3" s="3" t="n"/>
       <c r="K3" s="3" t="n"/>
-      <c r="L3" s="3" t="n"/>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t>Five years commencing 1973-01-13</t>
+          <t>5 years commencing 1973-01-13</t>
         </is>
       </c>
       <c r="N3" s="3" t="n"/>
@@ -3294,20 +5148,24 @@
       <c r="P3" s="3" t="n"/>
       <c r="Q3" s="3" t="inlineStr">
         <is>
-          <t>502/267; 872/279 exclusion</t>
-        </is>
-      </c>
-      <c r="R3" s="3" t="n"/>
+          <t>502/267; excluded from 872/279 to extent previously assigned</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Union ORRIs under 502/267</t>
+        </is>
+      </c>
       <c r="S3" s="3" t="n"/>
       <c r="T3" s="3" t="n"/>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V3" s="3" t="inlineStr">
         <is>
-          <t>Original OGL direct image</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W3" s="3" t="n">
@@ -3315,7 +5173,7 @@
       </c>
       <c r="X3" s="3" t="inlineStr">
         <is>
-          <t>HBP, amendments, releases, and modern linkage open</t>
+          <t>Images 1197–1198 and 4392. Instrument also covers 80 acres in Section 28; only 160 Section 32 row acres counted.</t>
         </is>
       </c>
     </row>
@@ -3332,7 +5190,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -3340,8 +5198,16 @@
           <t>1976-04-29</t>
         </is>
       </c>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>1976-06-09</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2991</t>
+        </is>
+      </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
           <t>307/31</t>
@@ -3357,8 +5223,16 @@
       </c>
       <c r="J4" s="3" t="n"/>
       <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>1/8</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1976-09-23</t>
+        </is>
+      </c>
       <c r="N4" s="3" t="n"/>
       <c r="O4" s="3" t="n"/>
       <c r="P4" s="3" t="n"/>
@@ -3367,25 +5241,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R4" s="3" t="n"/>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S4" s="3" t="n"/>
       <c r="T4" s="3" t="n"/>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V4" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W4" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X4" s="3" t="inlineStr">
         <is>
-          <t>Overlaps other rows; original OGL not reviewed</t>
+          <t>Images 1372 and 4391. Overlaps other listed rows; no present status or HBP inference.</t>
         </is>
       </c>
     </row>
@@ -3397,12 +5275,12 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Gertrude L. LaFortune et al., co-trustees</t>
+          <t>Gertrude L. LaFortune; Jeanne L. Fair; Mary Ann L. Wilcox; J.A. LaFortune Jr.; Robert J. LaFortune, co-trustees under the will of Joseph A. LaFortune</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -3427,8 +5305,16 @@
       </c>
       <c r="J5" s="3" t="n"/>
       <c r="K5" s="3" t="n"/>
-      <c r="L5" s="3" t="n"/>
-      <c r="M5" s="3" t="n"/>
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1977-11-28</t>
+        </is>
+      </c>
       <c r="N5" s="3" t="n"/>
       <c r="O5" s="3" t="n"/>
       <c r="P5" s="3" t="n"/>
@@ -3437,25 +5323,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R5" s="3" t="n"/>
+      <c r="R5" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S5" s="3" t="n"/>
       <c r="T5" s="3" t="n"/>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V5" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W5" s="3" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="X5" s="3" t="inlineStr">
         <is>
-          <t>Relationship to 340/304 open</t>
+          <t>Images 1522–1523 and 4391. Relationship to separate 340/304 remains open.</t>
         </is>
       </c>
     </row>
@@ -3472,7 +5362,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -3497,8 +5387,16 @@
       </c>
       <c r="J6" s="3" t="n"/>
       <c r="K6" s="3" t="n"/>
-      <c r="L6" s="3" t="n"/>
-      <c r="M6" s="3" t="n"/>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1977-11-28</t>
+        </is>
+      </c>
       <c r="N6" s="3" t="n"/>
       <c r="O6" s="3" t="n"/>
       <c r="P6" s="3" t="n"/>
@@ -3507,25 +5405,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R6" s="3" t="n"/>
+      <c r="R6" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S6" s="3" t="n"/>
       <c r="T6" s="3" t="n"/>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V6" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W6" s="3" t="n">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="X6" s="3" t="inlineStr">
         <is>
-          <t>Possible separate/corrective lease; do not double count</t>
+          <t>Images 1524–1525 and 4391. Separate overlapping lease; do not double count.</t>
         </is>
       </c>
     </row>
@@ -3542,7 +5444,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -3550,7 +5452,11 @@
           <t>1977-09-29</t>
         </is>
       </c>
-      <c r="E7" s="3" t="n"/>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>1977-11-07</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="n"/>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -3567,8 +5473,16 @@
       </c>
       <c r="J7" s="3" t="n"/>
       <c r="K7" s="3" t="n"/>
-      <c r="L7" s="3" t="n"/>
-      <c r="M7" s="3" t="n"/>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1977-11-27</t>
+        </is>
+      </c>
       <c r="N7" s="3" t="n"/>
       <c r="O7" s="3" t="n"/>
       <c r="P7" s="3" t="n"/>
@@ -3577,25 +5491,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R7" s="3" t="n"/>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S7" s="3" t="n"/>
       <c r="T7" s="3" t="n"/>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V7" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W7" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X7" s="3" t="inlineStr">
         <is>
-          <t>Overlapping legal</t>
+          <t>Images 1526–1527 and 4391. This is the only listed lease aliquot covering N/2 NW/4.</t>
         </is>
       </c>
     </row>
@@ -3612,7 +5530,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -3620,8 +5538,16 @@
           <t>1977-09-29</t>
         </is>
       </c>
-      <c r="E8" s="3" t="n"/>
-      <c r="F8" s="3" t="n"/>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1978-02-09</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>1089</t>
+        </is>
+      </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
           <t>342/564</t>
@@ -3637,8 +5563,16 @@
       </c>
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="3" t="n"/>
-      <c r="L8" s="3" t="n"/>
-      <c r="M8" s="3" t="n"/>
+      <c r="L8" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1977-11-30</t>
+        </is>
+      </c>
       <c r="N8" s="3" t="n"/>
       <c r="O8" s="3" t="n"/>
       <c r="P8" s="3" t="n"/>
@@ -3647,25 +5581,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R8" s="3" t="n"/>
+      <c r="R8" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S8" s="3" t="n"/>
       <c r="T8" s="3" t="n"/>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V8" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W8" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X8" s="3" t="inlineStr">
         <is>
-          <t>Overlapping legal</t>
+          <t>Images 1542–1543 and 4391. Overlapping legal; current status open.</t>
         </is>
       </c>
     </row>
@@ -3682,7 +5620,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -3690,8 +5628,16 @@
           <t>1977-11-01</t>
         </is>
       </c>
-      <c r="E9" s="3" t="n"/>
-      <c r="F9" s="3" t="n"/>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>1978-02-09</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>1090</t>
+        </is>
+      </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
           <t>342/566</t>
@@ -3707,8 +5653,16 @@
       </c>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="3" t="n"/>
-      <c r="L9" s="3" t="n"/>
-      <c r="M9" s="3" t="n"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>5 years commencing 1977-11-30</t>
+        </is>
+      </c>
       <c r="N9" s="3" t="n"/>
       <c r="O9" s="3" t="n"/>
       <c r="P9" s="3" t="n"/>
@@ -3717,25 +5671,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R9" s="3" t="n"/>
+      <c r="R9" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S9" s="3" t="n"/>
       <c r="T9" s="3" t="n"/>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V9" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W9" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X9" s="3" t="inlineStr">
         <is>
-          <t>Overlapping legal</t>
+          <t>Images 1544–1545 and 4391. Overlapping legal; current status open.</t>
         </is>
       </c>
     </row>
@@ -3752,7 +5710,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
@@ -3760,8 +5718,16 @@
           <t>1978-05-16</t>
         </is>
       </c>
-      <c r="E10" s="3" t="n"/>
-      <c r="F10" s="3" t="n"/>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>1978-06-27</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>5169</t>
+        </is>
+      </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
           <t>352/719</t>
@@ -3777,8 +5743,16 @@
       </c>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="3" t="n"/>
-      <c r="L10" s="3" t="n"/>
-      <c r="M10" s="3" t="n"/>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
       <c r="N10" s="3" t="n"/>
       <c r="O10" s="3" t="n"/>
       <c r="P10" s="3" t="n"/>
@@ -3787,25 +5761,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R10" s="3" t="n"/>
+      <c r="R10" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S10" s="3" t="n"/>
       <c r="T10" s="3" t="n"/>
       <c r="U10" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V10" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W10" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X10" s="3" t="inlineStr">
         <is>
-          <t>Overlapping legal</t>
+          <t>Images 1552–1553 and 4391. Face instrument 5169 conflicts with protocol index 5051; clerk confirmation required.</t>
         </is>
       </c>
     </row>
@@ -3822,7 +5800,7 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
@@ -3830,8 +5808,16 @@
           <t>1978-05-16</t>
         </is>
       </c>
-      <c r="E11" s="3" t="n"/>
-      <c r="F11" s="3" t="n"/>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>1978-06-27</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>5168</t>
+        </is>
+      </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
           <t>352/721</t>
@@ -3847,8 +5833,16 @@
       </c>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="3" t="n"/>
-      <c r="L11" s="3" t="n"/>
-      <c r="M11" s="3" t="n"/>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
       <c r="N11" s="3" t="n"/>
       <c r="O11" s="3" t="n"/>
       <c r="P11" s="3" t="n"/>
@@ -3857,25 +5851,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R11" s="3" t="n"/>
+      <c r="R11" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S11" s="3" t="n"/>
       <c r="T11" s="3" t="n"/>
       <c r="U11" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V11" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W11" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X11" s="3" t="inlineStr">
         <is>
-          <t>Overlapping legal</t>
+          <t>Images 1554–1555 and 4392. Face instrument 5168 conflicts with protocol index 5052; clerk confirmation required.</t>
         </is>
       </c>
     </row>
@@ -3887,12 +5885,12 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Great Western Oil &amp; Gas, Inc.</t>
+          <t>Great Western Oil &amp; Gas, Inc., a California corporation</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Union</t>
+          <t>Union Oil Company of California</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -3900,8 +5898,16 @@
           <t>1979-03-21</t>
         </is>
       </c>
-      <c r="E12" s="3" t="n"/>
-      <c r="F12" s="3" t="n"/>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>1979-04-30</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>3757</t>
+        </is>
+      </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
           <t>376/369</t>
@@ -3917,8 +5923,16 @@
       </c>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="3" t="n"/>
-      <c r="L12" s="3" t="n"/>
-      <c r="M12" s="3" t="n"/>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>3/16</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr">
+        <is>
+          <t>5 years</t>
+        </is>
+      </c>
       <c r="N12" s="3" t="n"/>
       <c r="O12" s="3" t="n"/>
       <c r="P12" s="3" t="n"/>
@@ -3927,25 +5941,29 @@
           <t>872/279</t>
         </is>
       </c>
-      <c r="R12" s="3" t="n"/>
+      <c r="R12" s="3" t="inlineStr">
+        <is>
+          <t>Union depth-limited ORRIs under 872/279</t>
+        </is>
+      </c>
       <c r="S12" s="3" t="n"/>
       <c r="T12" s="3" t="n"/>
       <c r="U12" s="3" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>OPEN_UNVERIFIED_CURRENT</t>
         </is>
       </c>
       <c r="V12" s="3" t="inlineStr">
         <is>
-          <t>Lease schedule reference</t>
+          <t>DIRECT ORIGINAL IMAGE + RECORDED EXHIBIT</t>
         </is>
       </c>
       <c r="W12" s="3" t="n">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="X12" s="3" t="inlineStr">
         <is>
-          <t>Correction metadata at 1039/20–23 unreviewed</t>
+          <t>Images 1569–1570 and 4392. Face instrument 3757 conflicts with protocol index 3707; correction metadata at 1039/20–23 remains unreviewed.</t>
         </is>
       </c>
     </row>
@@ -3957,6 +5975,117 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="33" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Acres</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Basis / Limitation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Row acres</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>1360</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Sum of the 11 Section 32 lease-row aliquots; only 160 Section 32 acres counted for 264/345</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Unique nominal acres</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>560</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Union of listed aliquots: NE/4, SE/4, SW/4, and N/2 NW/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Overlap</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>800</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>1,360 row acres minus 560 unique nominal acres</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Schedule gap</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>80</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>S/2 NW/4 is not among the Bk 872/Pg 279 listed lease aliquots</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Diversified net leasehold acres</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>NOT DETERMINED; document-location math does not prove current title, HBP, or quantum</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4488,16 +6617,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
@@ -4576,7 +6705,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T5 / exact tract allocation open</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -4611,166 +6740,14 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>T2</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>Diversified Production LLC — schedule-dependent claimant only</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>OK48147.001.1</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
-      <c r="E3" s="3" t="n"/>
-      <c r="F3" s="3" t="n"/>
-      <c r="G3" s="3" t="n"/>
-      <c r="H3" s="3" t="n"/>
-      <c r="I3" s="3" t="n"/>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>NOT DETERMINED</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>2395/462; 2400/566</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Obtain operative schedules and predecessor title</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>T3</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Diversified Production LLC — schedule-dependent claimant only</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>OK48147.001.1</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>NOT DETERMINED</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>2395/462; 2400/566</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr">
-        <is>
-          <t>Obtain operative schedules and predecessor title</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t>T4</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="inlineStr">
-        <is>
-          <t>Diversified Production LLC — schedule-dependent claimant only</t>
-        </is>
-      </c>
-      <c r="C5" s="3" t="inlineStr">
-        <is>
-          <t>OK48147.001.1</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-      <c r="H5" s="3" t="n"/>
-      <c r="I5" s="3" t="n"/>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>NOT DETERMINED</t>
-        </is>
-      </c>
-      <c r="K5" s="3" t="inlineStr">
-        <is>
-          <t>2395/462; 2400/566</t>
-        </is>
-      </c>
-      <c r="L5" s="3" t="inlineStr">
-        <is>
-          <t>Obtain operative schedules and predecessor title</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>T5</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Diversified Production LLC — schedule-dependent claimant only</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>OK48147.001.1</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n"/>
-      <c r="E6" s="3" t="n"/>
-      <c r="F6" s="3" t="n"/>
-      <c r="G6" s="3" t="n"/>
-      <c r="H6" s="3" t="n"/>
-      <c r="I6" s="3" t="n"/>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>NOT DETERMINED</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>2395/462; 2400/566</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr">
-        <is>
-          <t>Obtain operative schedules and predecessor title</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:L6"/>
+  <autoFilter ref="A1:L2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5298,103 +7275,4 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:G2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="26" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Party</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Recorded Address</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Normalized Address</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Address Type</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Effective/Recording Date</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Currentness Caveat</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Diversified Production LLC</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>1600 Corporate Drive, Birmingham, AL 35242</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>1600 Corporate Drive, Birmingham, AL 35242</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Recorded instrument address</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>2395/415–464; 2400/551–567</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>2022-11-18 / 2023-03-02</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Historic recorded address; not represented as verified current</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:G2"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToWidth="1"/>
-</worksheet>
 </file>
</xml_diff>